<commit_message>
🤖 Alerta diaria automática
</commit_message>
<xml_diff>
--- a/Alerta_Fiscalia.xlsx
+++ b/Alerta_Fiscalia.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,90 +467,6 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>URL_NOTICIA</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>1067962652</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>🟠 ALERTA MEDIA (3 Palabras)</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>JOSE FRANCISCO CHAVEZ SUAREZ</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>JOSE FRANCISCO SUAREZ</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>75.0%</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>2026-04-24</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>FEMINICIDIO AGRAVADO</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>https://www.fiscalia.gov.co/colombia/noticias/sentido-de-fallo-condenatorio-contra-senalado-responsable-de-crimen-de-su-pareja-en-el-sur-de-bogota/</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>1110459415</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>🟠 ALERTA MEDIA (3 Palabras)</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>JOSE FRANCISCO SUAREZ CAMACHO</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>JOSE FRANCISCO SUAREZ</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>75.0%</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>2026-04-24</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>FEMINICIDIO AGRAVADO</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>https://www.fiscalia.gov.co/colombia/noticias/sentido-de-fallo-condenatorio-contra-senalado-responsable-de-crimen-de-su-pareja-en-el-sur-de-bogota/</t>
         </is>
       </c>
     </row>

</xml_diff>